<commit_message>
Stamp the tracker with its version, and say so when one is old
The sheet now carries its version in cell A1 of Positions, because filenames get
renamed and cells do not. Distributed copies are named with the version too.

A tracker carrying none of the newer optional columns now gets a plain note on
load saying it is an older one, that it still works, and that nothing typed is
wasted. A holder hit exactly this and had no way to tell her sheet predated the
columns the tool was looking for.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracker-template.xlsx
+++ b/tracker-template.xlsx
@@ -762,13 +762,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A2:B42"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="24" min="1" max="1"/>
     <col width="104" customWidth="1" style="24" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="24.45" customHeight="1" s="25">
       <c r="B2" s="26" t="inlineStr">
         <is>
@@ -783,6 +784,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="17" customHeight="1" s="25">
       <c r="B5" s="28" t="inlineStr">
         <is>
@@ -797,6 +799,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="17" customHeight="1" s="25">
       <c r="B8" s="28" t="inlineStr">
         <is>
@@ -839,6 +842,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="17" customHeight="1" s="25">
       <c r="B15" s="28" t="inlineStr">
         <is>
@@ -888,6 +892,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="17" customHeight="1" s="25">
       <c r="B23" s="28" t="inlineStr">
         <is>
@@ -909,6 +914,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27" ht="15" customHeight="1" s="25">
       <c r="B27" s="33" t="inlineStr">
         <is>
@@ -916,6 +922,7 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="24" t="inlineStr">
         <is>
@@ -930,6 +937,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="24" t="inlineStr">
         <is>
@@ -944,6 +952,7 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="24" t="inlineStr">
         <is>
@@ -958,6 +967,7 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="24" t="inlineStr">
         <is>
@@ -972,15 +982,16 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="24" t="inlineStr">
         <is>
           <t>Fund or Single deal</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="24" t="inlineStr">
         <is>
           <t>Type "Fund" if the position holds several underlying investments, or "Single deal" if it is one company or one property. This is the simplest way to tell the tool how a position pays out: a fund sells down over several years, a single deal is bought on one date. It beats anything the tool would otherwise guess, including the Deals in fund count. If you leave it blank the tool still works out a sensible answer, but saying it outright is better.</t>
         </is>
@@ -1023,7 +1034,7 @@
     <row r="1" ht="16.15" customHeight="1" s="25">
       <c r="A1" s="34" t="inlineStr">
         <is>
-          <t>Positions  —  fill in the yellow cells, one row per deal</t>
+          <t>Positions  —  fill in the yellow cells, one row per deal        TRACKER v1.6</t>
         </is>
       </c>
     </row>
@@ -2043,7 +2054,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="15" customHeight="1" s="25">
       <c r="A18" s="48" t="inlineStr">
         <is>
@@ -2062,7 +2072,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="15" customHeight="1" s="25">
       <c r="A20" s="48" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
v1.16: IRR by deal, asset class and scenario, and a Marked Up MOIC column
Two features that ship together because they collide. IRR counts cash only; the markup is
the first paper figure the tool has held. The boundary is tested rather than intended.

A portfolio IRR pools the cash flows and solves once per simulated future, then ranks.
Averaging the thirteen deals instead gives a median of -5.4% against the correct 12.4%.

Diversification is now a number: every venture SPV has a ~30% chance of returning nothing
and a median IRR of 0.0%, but pooled as a sleeve the median is 7.2%.

A sponsor's multiple was invisible below the 90th percentile, so four deals with multiples
from 5.5x to 14.2x printed an identical 10.5%. The new sponsor-case column separates them.

A tracker that leaves the new column blank produces numbers identical to the ones it
produced before this version, verified against a frozen snapshot of the whole output.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracker-template.xlsx
+++ b/tracker-template.xlsx
@@ -762,14 +762,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A2:B42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="24" min="1" max="1"/>
     <col width="104" customWidth="1" style="24" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="24.45" customHeight="1" s="25">
       <c r="B2" s="26" t="inlineStr">
         <is>
@@ -784,7 +783,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="17" customHeight="1" s="25">
       <c r="B5" s="28" t="inlineStr">
         <is>
@@ -799,7 +797,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="17" customHeight="1" s="25">
       <c r="B8" s="28" t="inlineStr">
         <is>
@@ -842,7 +839,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="17" customHeight="1" s="25">
       <c r="B15" s="28" t="inlineStr">
         <is>
@@ -892,7 +888,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="17" customHeight="1" s="25">
       <c r="B23" s="28" t="inlineStr">
         <is>
@@ -914,7 +909,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27" ht="15" customHeight="1" s="25">
       <c r="B27" s="33" t="inlineStr">
         <is>
@@ -922,7 +916,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="24" t="inlineStr">
         <is>
@@ -937,7 +930,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="24" t="inlineStr">
         <is>
@@ -952,7 +944,6 @@
         </is>
       </c>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="24" t="inlineStr">
         <is>
@@ -967,7 +958,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="24" t="inlineStr">
         <is>
@@ -982,7 +972,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="24" t="inlineStr">
         <is>
@@ -1010,7 +999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="24" min="1" max="1"/>
@@ -1029,12 +1018,13 @@
     <col width="14" customWidth="1" style="25" min="18" max="18"/>
     <col width="46" customWidth="1" style="25" min="19" max="19"/>
     <col width="18" customWidth="1" style="25" min="20" max="20"/>
+    <col width="15" customWidth="1" style="25" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="16.15" customHeight="1" s="25">
       <c r="A1" s="34" t="inlineStr">
         <is>
-          <t>Positions  —  fill in the yellow cells, one row per deal        TRACKER v1.6</t>
+          <t>Positions  ·  fill in the yellow cells, one row per deal        TRACKER v1.7</t>
         </is>
       </c>
     </row>
@@ -1139,6 +1129,11 @@
           <t>Fund or Single deal</t>
         </is>
       </c>
+      <c r="U2" s="36" t="inlineStr">
+        <is>
+          <t>Marked Up MOIC</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="25">
       <c r="A3" s="37" t="inlineStr">
@@ -1151,11 +1146,7 @@
           <t>Income</t>
         </is>
       </c>
-      <c r="C3" s="37" t="inlineStr">
-        <is>
-          <t>Real Estate</t>
-        </is>
-      </c>
+      <c r="C3" s="37" t="n"/>
       <c r="D3" s="38" t="n">
         <v>50000</v>
       </c>
@@ -1169,50 +1160,37 @@
       <c r="G3" s="45" t="n">
         <v>2025</v>
       </c>
-      <c r="H3" s="45" t="n">
-        <v>5</v>
-      </c>
-      <c r="I3" s="41" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="J3" s="42" t="n">
-        <v>1.8</v>
-      </c>
+      <c r="H3" s="45" t="n"/>
+      <c r="I3" s="41" t="n"/>
+      <c r="J3" s="42" t="n"/>
       <c r="K3" s="37" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="L3" s="43">
-        <f>M3-MIN(3,MAX(1,ROUND(H3*0.3,0)))</f>
+        <f>IF(M3="","",M3-MIN(3,MAX(1,ROUND(H3*0.3,0))))</f>
         <v/>
       </c>
       <c r="M3" s="43">
-        <f>IF(O3&lt;&gt;"",O3,G3+H3)</f>
+        <f>IF(O3&lt;&gt;"",O3,IF(H3="","",G3+H3))</f>
         <v/>
       </c>
       <c r="N3" s="43">
-        <f>M3+2</f>
+        <f>IF(M3="","",M3+2)</f>
         <v/>
       </c>
       <c r="O3" s="44" t="n"/>
       <c r="P3" s="45" t="n"/>
-      <c r="Q3" s="45" t="n">
-        <v>4</v>
-      </c>
-      <c r="R3" s="45" t="n">
-        <v>6</v>
-      </c>
+      <c r="Q3" s="45" t="n"/>
+      <c r="R3" s="45" t="n"/>
       <c r="S3" s="37" t="inlineStr">
         <is>
           <t>Income floor. Quarterly cash I can plan a year around, with an equity kicker on the sale.</t>
         </is>
       </c>
-      <c r="T3" s="37" t="inlineStr">
-        <is>
-          <t>Fund</t>
-        </is>
-      </c>
+      <c r="T3" s="37" t="n"/>
+      <c r="U3" s="42" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1" s="25">
       <c r="A4" s="37" t="inlineStr">
@@ -1225,11 +1203,7 @@
           <t>Income</t>
         </is>
       </c>
-      <c r="C4" s="37" t="inlineStr">
-        <is>
-          <t>Real Estate</t>
-        </is>
-      </c>
+      <c r="C4" s="37" t="n"/>
       <c r="D4" s="38" t="n">
         <v>50000</v>
       </c>
@@ -1243,46 +1217,33 @@
       <c r="G4" s="45" t="n">
         <v>2026</v>
       </c>
-      <c r="H4" s="45" t="n">
-        <v>5</v>
-      </c>
-      <c r="I4" s="41" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="J4" s="42" t="n">
-        <v>1.75</v>
-      </c>
+      <c r="H4" s="45" t="n"/>
+      <c r="I4" s="41" t="n"/>
+      <c r="J4" s="42" t="n"/>
       <c r="K4" s="37" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="L4" s="43">
-        <f>M4-MIN(3,MAX(1,ROUND(H4*0.3,0)))</f>
+        <f>IF(M4="","",M4-MIN(3,MAX(1,ROUND(H4*0.3,0))))</f>
         <v/>
       </c>
       <c r="M4" s="43">
-        <f>IF(O4&lt;&gt;"",O4,G4+H4)</f>
+        <f>IF(O4&lt;&gt;"",O4,IF(H4="","",G4+H4))</f>
         <v/>
       </c>
       <c r="N4" s="43">
-        <f>M4+2</f>
+        <f>IF(M4="","",M4+2)</f>
         <v/>
       </c>
       <c r="O4" s="44" t="n"/>
       <c r="P4" s="45" t="n"/>
-      <c r="Q4" s="45" t="n">
-        <v>4</v>
-      </c>
-      <c r="R4" s="45" t="n">
-        <v>6</v>
-      </c>
+      <c r="Q4" s="45" t="n"/>
+      <c r="R4" s="45" t="n"/>
       <c r="S4" s="37" t="n"/>
-      <c r="T4" s="37" t="inlineStr">
-        <is>
-          <t>Fund</t>
-        </is>
-      </c>
+      <c r="T4" s="37" t="n"/>
+      <c r="U4" s="42" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="25">
       <c r="A5" s="37" t="inlineStr">
@@ -1295,11 +1256,7 @@
           <t>Income</t>
         </is>
       </c>
-      <c r="C5" s="37" t="inlineStr">
-        <is>
-          <t>Private Equity</t>
-        </is>
-      </c>
+      <c r="C5" s="37" t="n"/>
       <c r="D5" s="38" t="n">
         <v>50000</v>
       </c>
@@ -1313,44 +1270,33 @@
       <c r="G5" s="45" t="n">
         <v>2025</v>
       </c>
-      <c r="H5" s="45" t="n">
-        <v>7</v>
-      </c>
-      <c r="I5" s="41" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="J5" s="42" t="n">
-        <v>2.65</v>
-      </c>
+      <c r="H5" s="45" t="n"/>
+      <c r="I5" s="41" t="n"/>
+      <c r="J5" s="42" t="n"/>
       <c r="K5" s="37" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="L5" s="43">
-        <f>M5-MIN(3,MAX(1,ROUND(H5*0.3,0)))</f>
+        <f>IF(M5="","",M5-MIN(3,MAX(1,ROUND(H5*0.3,0))))</f>
         <v/>
       </c>
       <c r="M5" s="43">
-        <f>IF(O5&lt;&gt;"",O5,G5+H5)</f>
+        <f>IF(O5&lt;&gt;"",O5,IF(H5="","",G5+H5))</f>
         <v/>
       </c>
       <c r="N5" s="43">
-        <f>M5+2</f>
+        <f>IF(M5="","",M5+2)</f>
         <v/>
       </c>
       <c r="O5" s="44" t="n"/>
-      <c r="P5" s="45" t="n">
-        <v>1</v>
-      </c>
+      <c r="P5" s="45" t="n"/>
       <c r="Q5" s="45" t="n"/>
       <c r="R5" s="45" t="n"/>
       <c r="S5" s="37" t="n"/>
-      <c r="T5" s="37" t="inlineStr">
-        <is>
-          <t>Single deal</t>
-        </is>
-      </c>
+      <c r="T5" s="37" t="n"/>
+      <c r="U5" s="42" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="25">
       <c r="A6" s="37" t="inlineStr">
@@ -1363,11 +1309,7 @@
           <t>Income</t>
         </is>
       </c>
-      <c r="C6" s="37" t="inlineStr">
-        <is>
-          <t>Private Equity</t>
-        </is>
-      </c>
+      <c r="C6" s="37" t="n"/>
       <c r="D6" s="38" t="n">
         <v>50000</v>
       </c>
@@ -1381,44 +1323,33 @@
       <c r="G6" s="45" t="n">
         <v>2026</v>
       </c>
-      <c r="H6" s="45" t="n">
-        <v>7</v>
-      </c>
-      <c r="I6" s="41" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="J6" s="42" t="n">
-        <v>2.65</v>
-      </c>
+      <c r="H6" s="45" t="n"/>
+      <c r="I6" s="41" t="n"/>
+      <c r="J6" s="42" t="n"/>
       <c r="K6" s="37" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="L6" s="43">
-        <f>M6-MIN(3,MAX(1,ROUND(H6*0.3,0)))</f>
+        <f>IF(M6="","",M6-MIN(3,MAX(1,ROUND(H6*0.3,0))))</f>
         <v/>
       </c>
       <c r="M6" s="43">
-        <f>IF(O6&lt;&gt;"",O6,G6+H6)</f>
+        <f>IF(O6&lt;&gt;"",O6,IF(H6="","",G6+H6))</f>
         <v/>
       </c>
       <c r="N6" s="43">
-        <f>M6+2</f>
+        <f>IF(M6="","",M6+2)</f>
         <v/>
       </c>
       <c r="O6" s="44" t="n"/>
-      <c r="P6" s="45" t="n">
-        <v>1</v>
-      </c>
+      <c r="P6" s="45" t="n"/>
       <c r="Q6" s="45" t="n"/>
       <c r="R6" s="45" t="n"/>
       <c r="S6" s="37" t="n"/>
-      <c r="T6" s="37" t="inlineStr">
-        <is>
-          <t>Single deal</t>
-        </is>
-      </c>
+      <c r="T6" s="37" t="n"/>
+      <c r="U6" s="42" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1" s="25">
       <c r="A7" s="37" t="inlineStr">
@@ -1431,11 +1362,7 @@
           <t>Income</t>
         </is>
       </c>
-      <c r="C7" s="37" t="inlineStr">
-        <is>
-          <t>Private Credit</t>
-        </is>
-      </c>
+      <c r="C7" s="37" t="n"/>
       <c r="D7" s="38" t="n">
         <v>100000</v>
       </c>
@@ -1449,50 +1376,37 @@
       <c r="G7" s="45" t="n">
         <v>2026</v>
       </c>
-      <c r="H7" s="45" t="n">
-        <v>8</v>
-      </c>
-      <c r="I7" s="41" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="J7" s="42" t="n">
-        <v>3.27</v>
-      </c>
+      <c r="H7" s="45" t="n"/>
+      <c r="I7" s="41" t="n"/>
+      <c r="J7" s="42" t="n"/>
       <c r="K7" s="37" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
       <c r="L7" s="43">
-        <f>M7-MIN(3,MAX(1,ROUND(H7*0.3,0)))</f>
+        <f>IF(M7="","",M7-MIN(3,MAX(1,ROUND(H7*0.3,0))))</f>
         <v/>
       </c>
       <c r="M7" s="43">
-        <f>IF(O7&lt;&gt;"",O7,G7+H7)</f>
+        <f>IF(O7&lt;&gt;"",O7,IF(H7="","",G7+H7))</f>
         <v/>
       </c>
       <c r="N7" s="43">
-        <f>M7+2</f>
+        <f>IF(M7="","",M7+2)</f>
         <v/>
       </c>
       <c r="O7" s="44" t="n"/>
       <c r="P7" s="45" t="n"/>
-      <c r="Q7" s="45" t="n">
-        <v>5</v>
-      </c>
-      <c r="R7" s="45" t="n">
-        <v>8</v>
-      </c>
+      <c r="Q7" s="45" t="n"/>
+      <c r="R7" s="45" t="n"/>
       <c r="S7" s="37" t="inlineStr">
         <is>
           <t>Highest coupon in the book and a credit-tilted base case. Sized for the income, not the kicker.</t>
         </is>
       </c>
-      <c r="T7" s="37" t="inlineStr">
-        <is>
-          <t>Fund</t>
-        </is>
-      </c>
+      <c r="T7" s="37" t="n"/>
+      <c r="U7" s="42" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="25">
       <c r="A8" s="37" t="inlineStr">
@@ -1505,11 +1419,7 @@
           <t>Venture</t>
         </is>
       </c>
-      <c r="C8" s="37" t="inlineStr">
-        <is>
-          <t>VC</t>
-        </is>
-      </c>
+      <c r="C8" s="37" t="n"/>
       <c r="D8" s="38" t="n">
         <v>250000</v>
       </c>
@@ -1523,34 +1433,28 @@
       <c r="G8" s="45" t="n">
         <v>2025</v>
       </c>
-      <c r="H8" s="45" t="n">
-        <v>10</v>
-      </c>
+      <c r="H8" s="45" t="n"/>
       <c r="I8" s="41" t="n"/>
-      <c r="J8" s="42" t="n">
-        <v>3.96</v>
-      </c>
+      <c r="J8" s="42" t="n"/>
       <c r="K8" s="37" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="L8" s="43">
-        <f>M8-MIN(3,MAX(1,ROUND(H8*0.3,0)))</f>
+        <f>IF(M8="","",M8-MIN(3,MAX(1,ROUND(H8*0.3,0))))</f>
         <v/>
       </c>
       <c r="M8" s="43">
-        <f>IF(O8&lt;&gt;"",O8,G8+H8)</f>
+        <f>IF(O8&lt;&gt;"",O8,IF(H8="","",G8+H8))</f>
         <v/>
       </c>
       <c r="N8" s="43">
-        <f>M8+2</f>
+        <f>IF(M8="","",M8+2)</f>
         <v/>
       </c>
       <c r="O8" s="44" t="n"/>
-      <c r="P8" s="45" t="n">
-        <v>40</v>
-      </c>
+      <c r="P8" s="45" t="n"/>
       <c r="Q8" s="45" t="n"/>
       <c r="R8" s="45" t="n"/>
       <c r="S8" s="37" t="inlineStr">
@@ -1558,11 +1462,8 @@
           <t>The only thing I own that can return many times what I put in. Sized so it can go badly.</t>
         </is>
       </c>
-      <c r="T8" s="37" t="inlineStr">
-        <is>
-          <t>Fund</t>
-        </is>
-      </c>
+      <c r="T8" s="37" t="n"/>
+      <c r="U8" s="42" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="25">
       <c r="A9" s="37" t="inlineStr">
@@ -1575,11 +1476,7 @@
           <t>Venture</t>
         </is>
       </c>
-      <c r="C9" s="37" t="inlineStr">
-        <is>
-          <t>VC</t>
-        </is>
-      </c>
+      <c r="C9" s="37" t="n"/>
       <c r="D9" s="38" t="n">
         <v>25000</v>
       </c>
@@ -1593,42 +1490,33 @@
       <c r="G9" s="45" t="n">
         <v>2025</v>
       </c>
-      <c r="H9" s="45" t="n">
-        <v>10</v>
-      </c>
+      <c r="H9" s="45" t="n"/>
       <c r="I9" s="41" t="n"/>
-      <c r="J9" s="42" t="n">
-        <v>4</v>
-      </c>
+      <c r="J9" s="42" t="n"/>
       <c r="K9" s="37" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="L9" s="43">
-        <f>M9-MIN(3,MAX(1,ROUND(H9*0.3,0)))</f>
+        <f>IF(M9="","",M9-MIN(3,MAX(1,ROUND(H9*0.3,0))))</f>
         <v/>
       </c>
       <c r="M9" s="43">
-        <f>IF(O9&lt;&gt;"",O9,G9+H9)</f>
+        <f>IF(O9&lt;&gt;"",O9,IF(H9="","",G9+H9))</f>
         <v/>
       </c>
       <c r="N9" s="43">
-        <f>M9+2</f>
+        <f>IF(M9="","",M9+2)</f>
         <v/>
       </c>
       <c r="O9" s="44" t="n"/>
-      <c r="P9" s="45" t="n">
-        <v>1</v>
-      </c>
+      <c r="P9" s="45" t="n"/>
       <c r="Q9" s="45" t="n"/>
       <c r="R9" s="45" t="n"/>
       <c r="S9" s="37" t="n"/>
-      <c r="T9" s="37" t="inlineStr">
-        <is>
-          <t>Single deal</t>
-        </is>
-      </c>
+      <c r="T9" s="37" t="n"/>
+      <c r="U9" s="42" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="25">
       <c r="A10" s="37" t="inlineStr">
@@ -1641,11 +1529,7 @@
           <t>Venture</t>
         </is>
       </c>
-      <c r="C10" s="37" t="inlineStr">
-        <is>
-          <t>VC</t>
-        </is>
-      </c>
+      <c r="C10" s="37" t="n"/>
       <c r="D10" s="38" t="n">
         <v>25000</v>
       </c>
@@ -1659,42 +1543,33 @@
       <c r="G10" s="45" t="n">
         <v>2026</v>
       </c>
-      <c r="H10" s="45" t="n">
-        <v>10</v>
-      </c>
+      <c r="H10" s="45" t="n"/>
       <c r="I10" s="41" t="n"/>
-      <c r="J10" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J10" s="42" t="n"/>
       <c r="K10" s="37" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="L10" s="43">
-        <f>M10-MIN(3,MAX(1,ROUND(H10*0.3,0)))</f>
+        <f>IF(M10="","",M10-MIN(3,MAX(1,ROUND(H10*0.3,0))))</f>
         <v/>
       </c>
       <c r="M10" s="43">
-        <f>IF(O10&lt;&gt;"",O10,G10+H10)</f>
+        <f>IF(O10&lt;&gt;"",O10,IF(H10="","",G10+H10))</f>
         <v/>
       </c>
       <c r="N10" s="43">
-        <f>M10+2</f>
+        <f>IF(M10="","",M10+2)</f>
         <v/>
       </c>
       <c r="O10" s="44" t="n"/>
-      <c r="P10" s="45" t="n">
-        <v>1</v>
-      </c>
+      <c r="P10" s="45" t="n"/>
       <c r="Q10" s="45" t="n"/>
       <c r="R10" s="45" t="n"/>
       <c r="S10" s="37" t="n"/>
-      <c r="T10" s="37" t="inlineStr">
-        <is>
-          <t>Single deal</t>
-        </is>
-      </c>
+      <c r="T10" s="37" t="n"/>
+      <c r="U10" s="42" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="25">
       <c r="A11" s="37" t="inlineStr">
@@ -1707,11 +1582,7 @@
           <t>Venture</t>
         </is>
       </c>
-      <c r="C11" s="37" t="inlineStr">
-        <is>
-          <t>VC</t>
-        </is>
-      </c>
+      <c r="C11" s="37" t="n"/>
       <c r="D11" s="38" t="n">
         <v>20000</v>
       </c>
@@ -1725,42 +1596,33 @@
       <c r="G11" s="45" t="n">
         <v>2025</v>
       </c>
-      <c r="H11" s="45" t="n">
-        <v>5</v>
-      </c>
+      <c r="H11" s="45" t="n"/>
       <c r="I11" s="41" t="n"/>
-      <c r="J11" s="42" t="n">
-        <v>5</v>
-      </c>
+      <c r="J11" s="42" t="n"/>
       <c r="K11" s="37" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
       <c r="L11" s="43">
-        <f>M11-MIN(3,MAX(1,ROUND(H11*0.3,0)))</f>
+        <f>IF(M11="","",M11-MIN(3,MAX(1,ROUND(H11*0.3,0))))</f>
         <v/>
       </c>
       <c r="M11" s="43">
-        <f>IF(O11&lt;&gt;"",O11,G11+H11)</f>
+        <f>IF(O11&lt;&gt;"",O11,IF(H11="","",G11+H11))</f>
         <v/>
       </c>
       <c r="N11" s="43">
-        <f>M11+2</f>
+        <f>IF(M11="","",M11+2)</f>
         <v/>
       </c>
       <c r="O11" s="44" t="n"/>
-      <c r="P11" s="45" t="n">
-        <v>1</v>
-      </c>
+      <c r="P11" s="45" t="n"/>
       <c r="Q11" s="45" t="n"/>
       <c r="R11" s="45" t="n"/>
       <c r="S11" s="37" t="n"/>
-      <c r="T11" s="37" t="inlineStr">
-        <is>
-          <t>Single deal</t>
-        </is>
-      </c>
+      <c r="T11" s="37" t="n"/>
+      <c r="U11" s="42" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="25">
       <c r="A12" s="37" t="inlineStr">
@@ -1773,11 +1635,7 @@
           <t>Venture</t>
         </is>
       </c>
-      <c r="C12" s="37" t="inlineStr">
-        <is>
-          <t>VC</t>
-        </is>
-      </c>
+      <c r="C12" s="37" t="n"/>
       <c r="D12" s="38" t="n">
         <v>20000</v>
       </c>
@@ -1791,42 +1649,33 @@
       <c r="G12" s="45" t="n">
         <v>2026</v>
       </c>
-      <c r="H12" s="45" t="n">
-        <v>10</v>
-      </c>
+      <c r="H12" s="45" t="n"/>
       <c r="I12" s="41" t="n"/>
-      <c r="J12" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J12" s="42" t="n"/>
       <c r="K12" s="37" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
       <c r="L12" s="43">
-        <f>M12-MIN(3,MAX(1,ROUND(H12*0.3,0)))</f>
+        <f>IF(M12="","",M12-MIN(3,MAX(1,ROUND(H12*0.3,0))))</f>
         <v/>
       </c>
       <c r="M12" s="43">
-        <f>IF(O12&lt;&gt;"",O12,G12+H12)</f>
+        <f>IF(O12&lt;&gt;"",O12,IF(H12="","",G12+H12))</f>
         <v/>
       </c>
       <c r="N12" s="43">
-        <f>M12+2</f>
+        <f>IF(M12="","",M12+2)</f>
         <v/>
       </c>
       <c r="O12" s="44" t="n"/>
-      <c r="P12" s="45" t="n">
-        <v>1</v>
-      </c>
+      <c r="P12" s="45" t="n"/>
       <c r="Q12" s="45" t="n"/>
       <c r="R12" s="45" t="n"/>
       <c r="S12" s="37" t="n"/>
-      <c r="T12" s="37" t="inlineStr">
-        <is>
-          <t>Single deal</t>
-        </is>
-      </c>
+      <c r="T12" s="37" t="n"/>
+      <c r="U12" s="42" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="25">
       <c r="A13" s="37" t="inlineStr">
@@ -1839,11 +1688,7 @@
           <t>Venture</t>
         </is>
       </c>
-      <c r="C13" s="37" t="inlineStr">
-        <is>
-          <t>VC</t>
-        </is>
-      </c>
+      <c r="C13" s="37" t="n"/>
       <c r="D13" s="38" t="n">
         <v>10000</v>
       </c>
@@ -1857,42 +1702,33 @@
       <c r="G13" s="45" t="n">
         <v>2025</v>
       </c>
-      <c r="H13" s="45" t="n">
-        <v>10</v>
-      </c>
+      <c r="H13" s="45" t="n"/>
       <c r="I13" s="41" t="n"/>
-      <c r="J13" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J13" s="42" t="n"/>
       <c r="K13" s="37" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
       <c r="L13" s="43">
-        <f>M13-MIN(3,MAX(1,ROUND(H13*0.3,0)))</f>
+        <f>IF(M13="","",M13-MIN(3,MAX(1,ROUND(H13*0.3,0))))</f>
         <v/>
       </c>
       <c r="M13" s="43">
-        <f>IF(O13&lt;&gt;"",O13,G13+H13)</f>
+        <f>IF(O13&lt;&gt;"",O13,IF(H13="","",G13+H13))</f>
         <v/>
       </c>
       <c r="N13" s="43">
-        <f>M13+2</f>
+        <f>IF(M13="","",M13+2)</f>
         <v/>
       </c>
       <c r="O13" s="44" t="n"/>
-      <c r="P13" s="45" t="n">
-        <v>1</v>
-      </c>
+      <c r="P13" s="45" t="n"/>
       <c r="Q13" s="45" t="n"/>
       <c r="R13" s="45" t="n"/>
       <c r="S13" s="37" t="n"/>
-      <c r="T13" s="37" t="inlineStr">
-        <is>
-          <t>Single deal</t>
-        </is>
-      </c>
+      <c r="T13" s="37" t="n"/>
+      <c r="U13" s="42" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="25">
       <c r="A14" s="37" t="inlineStr">
@@ -1905,11 +1741,7 @@
           <t>Venture</t>
         </is>
       </c>
-      <c r="C14" s="37" t="inlineStr">
-        <is>
-          <t>VC</t>
-        </is>
-      </c>
+      <c r="C14" s="37" t="n"/>
       <c r="D14" s="38" t="n">
         <v>10000</v>
       </c>
@@ -1923,42 +1755,33 @@
       <c r="G14" s="45" t="n">
         <v>2026</v>
       </c>
-      <c r="H14" s="45" t="n">
-        <v>10</v>
-      </c>
+      <c r="H14" s="45" t="n"/>
       <c r="I14" s="41" t="n"/>
-      <c r="J14" s="42" t="n">
-        <v>2.71</v>
-      </c>
+      <c r="J14" s="42" t="n"/>
       <c r="K14" s="37" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
       <c r="L14" s="43">
-        <f>M14-MIN(3,MAX(1,ROUND(H14*0.3,0)))</f>
+        <f>IF(M14="","",M14-MIN(3,MAX(1,ROUND(H14*0.3,0))))</f>
         <v/>
       </c>
       <c r="M14" s="43">
-        <f>IF(O14&lt;&gt;"",O14,G14+H14)</f>
+        <f>IF(O14&lt;&gt;"",O14,IF(H14="","",G14+H14))</f>
         <v/>
       </c>
       <c r="N14" s="43">
-        <f>M14+2</f>
+        <f>IF(M14="","",M14+2)</f>
         <v/>
       </c>
       <c r="O14" s="44" t="n"/>
-      <c r="P14" s="45" t="n">
-        <v>1</v>
-      </c>
+      <c r="P14" s="45" t="n"/>
       <c r="Q14" s="45" t="n"/>
       <c r="R14" s="45" t="n"/>
       <c r="S14" s="37" t="n"/>
-      <c r="T14" s="37" t="inlineStr">
-        <is>
-          <t>Single deal</t>
-        </is>
-      </c>
+      <c r="T14" s="37" t="n"/>
+      <c r="U14" s="42" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="25">
       <c r="A15" s="37" t="inlineStr">
@@ -1971,11 +1794,7 @@
           <t>Venture</t>
         </is>
       </c>
-      <c r="C15" s="37" t="inlineStr">
-        <is>
-          <t>VC</t>
-        </is>
-      </c>
+      <c r="C15" s="37" t="n"/>
       <c r="D15" s="38" t="n">
         <v>5000</v>
       </c>
@@ -1989,42 +1808,33 @@
       <c r="G15" s="45" t="n">
         <v>2025</v>
       </c>
-      <c r="H15" s="45" t="n">
-        <v>10</v>
-      </c>
+      <c r="H15" s="45" t="n"/>
       <c r="I15" s="41" t="n"/>
-      <c r="J15" s="42" t="n">
-        <v>1.78</v>
-      </c>
+      <c r="J15" s="42" t="n"/>
       <c r="K15" s="37" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
       <c r="L15" s="43">
-        <f>M15-MIN(3,MAX(1,ROUND(H15*0.3,0)))</f>
+        <f>IF(M15="","",M15-MIN(3,MAX(1,ROUND(H15*0.3,0))))</f>
         <v/>
       </c>
       <c r="M15" s="43">
-        <f>IF(O15&lt;&gt;"",O15,G15+H15)</f>
+        <f>IF(O15&lt;&gt;"",O15,IF(H15="","",G15+H15))</f>
         <v/>
       </c>
       <c r="N15" s="43">
-        <f>M15+2</f>
+        <f>IF(M15="","",M15+2)</f>
         <v/>
       </c>
       <c r="O15" s="44" t="n"/>
-      <c r="P15" s="45" t="n">
-        <v>1</v>
-      </c>
+      <c r="P15" s="45" t="n"/>
       <c r="Q15" s="45" t="n"/>
       <c r="R15" s="45" t="n"/>
       <c r="S15" s="37" t="n"/>
-      <c r="T15" s="37" t="inlineStr">
-        <is>
-          <t>Single deal</t>
-        </is>
-      </c>
+      <c r="T15" s="37" t="n"/>
+      <c r="U15" s="42" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="25">
       <c r="A16" s="46" t="inlineStr">
@@ -2072,6 +1882,13 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Hold, Coupon, Sponsor MOIC, Asset class and the fund columns are deliberately BLANK on these example rows. Those terms are identical for everyone who bought the deal, so they now live in one shared file per deal and the tool fills them in. Anything you type here overrides the shared file and nothing argues with you — which is why a figure typed before a sponsor corrected its terms is worth checking.</t>
+        </is>
+      </c>
+    </row>
     <row r="20" ht="15" customHeight="1" s="25">
       <c r="A20" s="48" t="inlineStr">
         <is>
@@ -2087,6 +1904,13 @@
       <c r="T20" s="37" t="inlineStr">
         <is>
           <t>Single deal</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Marked Up MOIC is optional. It records what you believe a position is worth now, and it drives a paper track shown beside the cash forecast rather than inside it. It never moves a cash figure and never enters the IRR.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v1.45: Asilia's second capital call is funded
Example book: Asilia GC Fund funded 24,000 / uncalled 76,000, next call Q1 2027 ~20,000.
Tracker template carries the same figures. No change to the model.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracker-template.xlsx
+++ b/tracker-template.xlsx
@@ -765,14 +765,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:B44"/>
+  <dimension ref="A2:B44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="24" min="1" max="1"/>
     <col width="104" customWidth="1" style="24" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="24.45" customHeight="1" s="25">
       <c r="B2" s="26" t="inlineStr">
         <is>
@@ -787,7 +786,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="17" customHeight="1" s="25">
       <c r="B5" s="28" t="inlineStr">
         <is>
@@ -802,7 +800,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="17" customHeight="1" s="25">
       <c r="B8" s="28" t="inlineStr">
         <is>
@@ -845,7 +842,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="17" customHeight="1" s="25">
       <c r="B15" s="28" t="inlineStr">
         <is>
@@ -895,7 +891,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="17" customHeight="1" s="25">
       <c r="B23" s="28" t="inlineStr">
         <is>
@@ -931,7 +926,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="B29" s="33" t="inlineStr">
         <is>
@@ -939,7 +933,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="24" t="inlineStr">
         <is>
@@ -954,7 +947,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="24" t="inlineStr">
         <is>
@@ -969,7 +961,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" s="24" t="inlineStr">
         <is>
@@ -984,7 +975,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="24" t="inlineStr">
         <is>
@@ -999,7 +989,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="24" t="inlineStr">
         <is>
@@ -1415,7 +1404,7 @@
         <v>100000</v>
       </c>
       <c r="E7" s="38" t="n">
-        <v>19000</v>
+        <v>24000</v>
       </c>
       <c r="F7" s="39">
         <f>MAX(0,D7-E7)</f>

</xml_diff>